<commit_message>
KB-15422: updated sample files
</commit_message>
<xml_diff>
--- a/MDO/client-assets/assets/common/user-bulk-creation-upload-sample/user-bulk-upload-sample.xlsx
+++ b/MDO/client-assets/assets/common/user-bulk-creation-upload-sample/user-bulk-upload-sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KB-iGot\Fork Repo\sunbird-cb-portal-assets\MDO\client-assets\assets\common\user-bulk-creation-upload-sample\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VikasBhardwaj\Downloads\Sample file Afzal\downloaded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C74520E-2CB1-4691-8771-76E807D1F37B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65D4F7FB-2A2C-4876-9A8C-036DD5EF8446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -296,9 +296,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -336,7 +336,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -442,7 +442,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -584,7 +584,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -593,25 +593,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q5"/>
-  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="28.44140625" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="21.109375" customWidth="1"/>
-    <col min="5" max="5" width="21.21875" customWidth="1"/>
-    <col min="6" max="6" width="11.21875" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" customWidth="1"/>
-    <col min="8" max="8" width="26.109375" customWidth="1"/>
-    <col min="9" max="9" width="13.109375" customWidth="1"/>
-    <col min="10" max="10" width="15.5546875" customWidth="1"/>
-    <col min="11" max="11" width="14.6640625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="23.6328125" customWidth="1"/>
+    <col min="2" max="2" width="28.453125" customWidth="1"/>
+    <col min="3" max="3" width="23.54296875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="21.08984375" customWidth="1"/>
+    <col min="5" max="5" width="21.1796875" customWidth="1"/>
+    <col min="6" max="6" width="11.1796875" customWidth="1"/>
+    <col min="7" max="7" width="10.54296875" customWidth="1"/>
+    <col min="8" max="8" width="26.08984375" customWidth="1"/>
+    <col min="9" max="9" width="13.08984375" customWidth="1"/>
+    <col min="10" max="10" width="15.54296875" customWidth="1"/>
+    <col min="11" max="11" width="14.6328125" style="4" customWidth="1"/>
     <col min="12" max="12" width="17" customWidth="1"/>
-    <col min="13" max="13" width="18.77734375" customWidth="1"/>
-    <col min="14" max="14" width="15.5546875" customWidth="1"/>
+    <col min="13" max="13" width="18.81640625" customWidth="1"/>
+    <col min="14" max="14" width="15.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>24</v>
       </c>
@@ -655,7 +655,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>26</v>
       </c>
@@ -686,6 +686,9 @@
       <c r="J2" t="s">
         <v>7</v>
       </c>
+      <c r="K2" s="5">
+        <v>201010</v>
+      </c>
       <c r="L2" t="s">
         <v>10</v>
       </c>
@@ -696,7 +699,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>27</v>
       </c>
@@ -743,7 +746,7 @@
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
@@ -774,7 +777,9 @@
       <c r="J4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="5"/>
+      <c r="K4" s="5">
+        <v>201010</v>
+      </c>
       <c r="L4" s="1" t="s">
         <v>10</v>
       </c>
@@ -788,7 +793,7 @@
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>29</v>
       </c>

</xml_diff>